<commit_message>
Update Relatório de Planejamento.xlsx
</commit_message>
<xml_diff>
--- a/xlsx/Relatório de Planejamento.xlsx
+++ b/xlsx/Relatório de Planejamento.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8980" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9043" uniqueCount="22">
   <si>
     <t>Resumo do Planejamento</t>
   </si>
@@ -739,26 +739,32 @@
       <c r="G22" s="7"/>
     </row>
     <row r="23">
-      <c r="B23" s="10"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
+      <c r="B23" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>7</v>
+      </c>
       <c r="E23" s="10"/>
       <c r="F23" s="11"/>
       <c r="G23" s="11"/>
     </row>
     <row r="24">
-      <c r="B24" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E24" s="6"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="13"/>
+      <c r="B24" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E24" s="10"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="11"/>
     </row>
     <row r="25">
       <c r="B25" s="7" t="s">
@@ -770,9 +776,9 @@
       <c r="D25" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="E25" s="14"/>
-      <c r="F25" s="7"/>
-      <c r="G25" s="7"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="11"/>
     </row>
     <row r="26">
       <c r="B26" s="7" t="s">
@@ -784,9 +790,9 @@
       <c r="D26" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="E26" s="14"/>
-      <c r="F26" s="7"/>
-      <c r="G26" s="7"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="11"/>
+      <c r="G26" s="11"/>
     </row>
     <row r="27">
       <c r="B27" s="7" t="s">
@@ -798,9 +804,9 @@
       <c r="D27" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="E27" s="14"/>
-      <c r="F27" s="7"/>
-      <c r="G27" s="7"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="11"/>
+      <c r="G27" s="11"/>
     </row>
     <row r="28">
       <c r="B28" s="7" t="s">
@@ -812,9 +818,9 @@
       <c r="D28" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="E28" s="14"/>
-      <c r="F28" s="7"/>
-      <c r="G28" s="7"/>
+      <c r="E28" s="10"/>
+      <c r="F28" s="11"/>
+      <c r="G28" s="11"/>
     </row>
     <row r="29">
       <c r="B29" s="7" t="s">
@@ -826,9 +832,9 @@
       <c r="D29" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="E29" s="14"/>
-      <c r="F29" s="7"/>
-      <c r="G29" s="7"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="11"/>
+      <c r="G29" s="11"/>
     </row>
     <row r="30">
       <c r="B30" s="7" t="s">
@@ -840,9 +846,9 @@
       <c r="D30" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="E30" s="14"/>
-      <c r="F30" s="7"/>
-      <c r="G30" s="7"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="11"/>
+      <c r="G30" s="11"/>
     </row>
     <row r="31">
       <c r="B31" s="7" t="s">
@@ -854,9 +860,9 @@
       <c r="D31" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="E31" s="14"/>
-      <c r="F31" s="7"/>
-      <c r="G31" s="7"/>
+      <c r="E31" s="10"/>
+      <c r="F31" s="11"/>
+      <c r="G31" s="11"/>
     </row>
     <row r="32">
       <c r="B32" s="7" t="s">
@@ -868,9 +874,9 @@
       <c r="D32" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="E32" s="14"/>
-      <c r="F32" s="7"/>
-      <c r="G32" s="7"/>
+      <c r="E32" s="10"/>
+      <c r="F32" s="11"/>
+      <c r="G32" s="11"/>
     </row>
     <row r="33">
       <c r="B33" s="7" t="s">
@@ -882,9 +888,9 @@
       <c r="D33" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="E33" s="14"/>
-      <c r="F33" s="7"/>
-      <c r="G33" s="7"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="11"/>
+      <c r="G33" s="11"/>
     </row>
     <row r="34">
       <c r="B34" s="7" t="s">
@@ -896,45 +902,45 @@
       <c r="D34" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="E34" s="14"/>
-      <c r="F34" s="7"/>
-      <c r="G34" s="7"/>
+      <c r="E34" s="10"/>
+      <c r="F34" s="11"/>
+      <c r="G34" s="11"/>
     </row>
     <row r="35">
-      <c r="B35" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C35" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D35" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="E35" s="14"/>
-      <c r="F35" s="7"/>
-      <c r="G35" s="7"/>
+      <c r="B35" s="10"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="10"/>
+      <c r="E35" s="10"/>
+      <c r="F35" s="11"/>
+      <c r="G35" s="11"/>
     </row>
     <row r="36">
-      <c r="B36" s="10"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="10"/>
-      <c r="F36" s="11"/>
-      <c r="G36" s="11"/>
+      <c r="B36" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E36" s="6"/>
+      <c r="F36" s="13"/>
+      <c r="G36" s="13"/>
     </row>
     <row r="37">
-      <c r="B37" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E37" s="6"/>
-      <c r="F37" s="13"/>
-      <c r="G37" s="13"/>
+      <c r="B37" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E37" s="14"/>
+      <c r="F37" s="7"/>
+      <c r="G37" s="7"/>
     </row>
     <row r="38">
       <c r="B38" s="7" t="s">
@@ -1203,32 +1209,26 @@
       <c r="G56" s="7"/>
     </row>
     <row r="57">
-      <c r="B57" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C57" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D57" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="E57" s="14"/>
-      <c r="F57" s="7"/>
-      <c r="G57" s="7"/>
+      <c r="B57" s="10"/>
+      <c r="C57" s="10"/>
+      <c r="D57" s="10"/>
+      <c r="E57" s="10"/>
+      <c r="F57" s="11"/>
+      <c r="G57" s="11"/>
     </row>
     <row r="58">
-      <c r="B58" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C58" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D58" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="E58" s="14"/>
-      <c r="F58" s="7"/>
-      <c r="G58" s="7"/>
+      <c r="B58" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C58" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D58" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E58" s="6"/>
+      <c r="F58" s="13"/>
+      <c r="G58" s="13"/>
     </row>
     <row r="59">
       <c r="B59" s="7" t="s">
@@ -42417,6 +42417,300 @@
       <c r="E3000" s="14"/>
       <c r="F3000" s="7"/>
       <c r="G3000" s="7"/>
+    </row>
+    <row r="3001">
+      <c r="B3001" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3001" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3001" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3001" s="14"/>
+      <c r="F3001" s="7"/>
+      <c r="G3001" s="7"/>
+    </row>
+    <row r="3002">
+      <c r="B3002" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3002" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3002" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3002" s="14"/>
+      <c r="F3002" s="7"/>
+      <c r="G3002" s="7"/>
+    </row>
+    <row r="3003">
+      <c r="B3003" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3003" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3003" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3003" s="14"/>
+      <c r="F3003" s="7"/>
+      <c r="G3003" s="7"/>
+    </row>
+    <row r="3004">
+      <c r="B3004" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3004" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3004" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3004" s="14"/>
+      <c r="F3004" s="7"/>
+      <c r="G3004" s="7"/>
+    </row>
+    <row r="3005">
+      <c r="B3005" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3005" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3005" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3005" s="14"/>
+      <c r="F3005" s="7"/>
+      <c r="G3005" s="7"/>
+    </row>
+    <row r="3006">
+      <c r="B3006" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3006" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3006" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3006" s="14"/>
+      <c r="F3006" s="7"/>
+      <c r="G3006" s="7"/>
+    </row>
+    <row r="3007">
+      <c r="B3007" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3007" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3007" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3007" s="14"/>
+      <c r="F3007" s="7"/>
+      <c r="G3007" s="7"/>
+    </row>
+    <row r="3008">
+      <c r="B3008" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3008" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3008" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3008" s="14"/>
+      <c r="F3008" s="7"/>
+      <c r="G3008" s="7"/>
+    </row>
+    <row r="3009">
+      <c r="B3009" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3009" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3009" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3009" s="14"/>
+      <c r="F3009" s="7"/>
+      <c r="G3009" s="7"/>
+    </row>
+    <row r="3010">
+      <c r="B3010" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3010" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3010" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3010" s="14"/>
+      <c r="F3010" s="7"/>
+      <c r="G3010" s="7"/>
+    </row>
+    <row r="3011">
+      <c r="B3011" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3011" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3011" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3011" s="14"/>
+      <c r="F3011" s="7"/>
+      <c r="G3011" s="7"/>
+    </row>
+    <row r="3012">
+      <c r="B3012" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3012" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3012" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3012" s="14"/>
+      <c r="F3012" s="7"/>
+      <c r="G3012" s="7"/>
+    </row>
+    <row r="3013">
+      <c r="B3013" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3013" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3013" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3013" s="14"/>
+      <c r="F3013" s="7"/>
+      <c r="G3013" s="7"/>
+    </row>
+    <row r="3014">
+      <c r="B3014" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3014" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3014" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3014" s="14"/>
+      <c r="F3014" s="7"/>
+      <c r="G3014" s="7"/>
+    </row>
+    <row r="3015">
+      <c r="B3015" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3015" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3015" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3015" s="14"/>
+      <c r="F3015" s="7"/>
+      <c r="G3015" s="7"/>
+    </row>
+    <row r="3016">
+      <c r="B3016" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3016" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3016" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3016" s="14"/>
+      <c r="F3016" s="7"/>
+      <c r="G3016" s="7"/>
+    </row>
+    <row r="3017">
+      <c r="B3017" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3017" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3017" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3017" s="14"/>
+      <c r="F3017" s="7"/>
+      <c r="G3017" s="7"/>
+    </row>
+    <row r="3018">
+      <c r="B3018" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3018" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3018" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3018" s="14"/>
+      <c r="F3018" s="7"/>
+      <c r="G3018" s="7"/>
+    </row>
+    <row r="3019">
+      <c r="B3019" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3019" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3019" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3019" s="14"/>
+      <c r="F3019" s="7"/>
+      <c r="G3019" s="7"/>
+    </row>
+    <row r="3020">
+      <c r="B3020" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3020" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3020" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3020" s="14"/>
+      <c r="F3020" s="7"/>
+      <c r="G3020" s="7"/>
+    </row>
+    <row r="3021">
+      <c r="B3021" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3021" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3021" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3021" s="14"/>
+      <c r="F3021" s="7"/>
+      <c r="G3021" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>